<commit_message>
Fig.7 (10 h): show only the three windows where things change (broken axis, 2-min bins), candidate change points marked; OLTP no-elimination explained (combos within 6.7% < 15%)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig7_10h.xlsx
+++ b/figs/data/fig7_10h.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="그림7 10시간 (10분 단위)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전환 직후 (1분 단위)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="① OLTP 시작 OLTP 시작" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② 전환 직후 전환 직후" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ 마지막 30분 마지막 30분" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -142,7 +143,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>(가) OLTP → Varmail 10시간: 10분 구간 WAF (낮을수록 좋음)</a:t>
+              <a:t>(가) OLTP → Varmail 10시간: 2분 구간 WAF (낮을수록 좋음)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -156,7 +157,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'그림7 10시간 (10분 단위)'!B1</f>
+              <f>'① OLTP 시작 OLTP 시작'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -184,12 +185,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$A$2:$A$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$A$2:$A$31</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$B$2:$B$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$B$2:$B$31</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -199,7 +200,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'그림7 10시간 (10분 단위)'!D1</f>
+              <f>'① OLTP 시작 OLTP 시작'!D1</f>
             </strRef>
           </tx>
           <spPr>
@@ -227,12 +228,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$C$2:$C$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$C$2:$C$29</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$D$2:$D$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$D$2:$D$29</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -244,7 +245,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="10.05"/>
+          <max val="1"/>
           <min val="0"/>
         </scaling>
         <delete val="0"/>
@@ -268,13 +269,13 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
-        <majorUnit val="1"/>
+        <majorUnit val="0.1"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="2.5"/>
+          <max val="1.6"/>
           <min val="1.2"/>
         </scaling>
         <delete val="0"/>
@@ -336,7 +337,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'그림7 10시간 (10분 단위)'!F1</f>
+              <f>'① OLTP 시작 OLTP 시작'!F1</f>
             </strRef>
           </tx>
           <spPr>
@@ -364,12 +365,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$E$2:$E$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$E$2:$E$31</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$F$2:$F$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$F$2:$F$31</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -381,7 +382,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="10.05"/>
+          <max val="1"/>
           <min val="0"/>
         </scaling>
         <delete val="0"/>
@@ -405,7 +406,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
-        <majorUnit val="1"/>
+        <majorUnit val="0.1"/>
       </valAx>
       <valAx>
         <axId val="20"/>
@@ -473,7 +474,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'그림7 10시간 (10분 단위)'!H1</f>
+              <f>'① OLTP 시작 OLTP 시작'!H1</f>
             </strRef>
           </tx>
           <spPr>
@@ -501,12 +502,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$G$2:$G$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$G$2:$G$31</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림7 10시간 (10분 단위)'!$H$2:$H$61</f>
+              <f>'① OLTP 시작 OLTP 시작'!$H$2:$H$31</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -518,7 +519,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="10.05"/>
+          <max val="1"/>
           <min val="0"/>
         </scaling>
         <delete val="0"/>
@@ -542,7 +543,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
-        <majorUnit val="1"/>
+        <majorUnit val="0.1"/>
       </valAx>
       <valAx>
         <axId val="20"/>
@@ -596,7 +597,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>(가) OLTP → Varmail 10시간: 1분 구간 WAF (낮을수록 좋음)</a:t>
+              <a:t>(가) OLTP → Varmail 10시간: 2분 구간 WAF (낮을수록 좋음)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -610,7 +611,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'전환 직후 (1분 단위)'!B1</f>
+              <f>'② 전환 직후 전환 직후'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -638,12 +639,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$A$2:$A$43</f>
+              <f>'② 전환 직후 전환 직후'!$A$2:$A$25</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$B$2:$B$43</f>
+              <f>'② 전환 직후 전환 직후'!$B$2:$B$25</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -653,7 +654,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'전환 직후 (1분 단위)'!D1</f>
+              <f>'② 전환 직후 전환 직후'!D1</f>
             </strRef>
           </tx>
           <spPr>
@@ -681,12 +682,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$C$2:$C$43</f>
+              <f>'② 전환 직후 전환 직후'!$C$2:$C$25</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$D$2:$D$43</f>
+              <f>'② 전환 직후 전환 직후'!$D$2:$D$25</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -698,7 +699,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="5.65"/>
+          <max val="5.75"/>
           <min val="4.95"/>
         </scaling>
         <delete val="0"/>
@@ -790,7 +791,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'전환 직후 (1분 단위)'!F1</f>
+              <f>'② 전환 직후 전환 직후'!F1</f>
             </strRef>
           </tx>
           <spPr>
@@ -818,12 +819,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$E$2:$E$43</f>
+              <f>'② 전환 직후 전환 직후'!$E$2:$E$25</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$F$2:$F$43</f>
+              <f>'② 전환 직후 전환 직후'!$F$2:$F$25</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -835,7 +836,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="5.65"/>
+          <max val="5.75"/>
           <min val="4.95"/>
         </scaling>
         <delete val="0"/>
@@ -927,7 +928,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'전환 직후 (1분 단위)'!H1</f>
+              <f>'② 전환 직후 전환 직후'!H1</f>
             </strRef>
           </tx>
           <spPr>
@@ -955,12 +956,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$G$2:$G$43</f>
+              <f>'② 전환 직후 전환 직후'!$G$2:$G$25</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'전환 직후 (1분 단위)'!$H$2:$H$43</f>
+              <f>'② 전환 직후 전환 직후'!$H$2:$H$25</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -972,8 +973,462 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="5.65"/>
+          <max val="5.75"/>
           <min val="4.95"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>측정 시작 후 시간 (시간)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+        <majorUnit val="0.1"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="48"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>남은 후보 수</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="span"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>(가) OLTP → Varmail 10시간: 2분 구간 WAF (낮을수록 좋음)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <scatterStyle val="lineMarker"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'③ 마지막 30분 마지막 30분'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="2A78D6"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$A$2:$A$15</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$B$2:$B$15</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'③ 마지막 30분 마지막 30분'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="E3A33B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="E3A33B"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="E3A33B"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$C$2:$C$16</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$D$2:$D$16</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="10.05"/>
+          <min val="9.550000000000001"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>측정 시작 후 시간 (시간)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+        <majorUnit val="0.1"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="2.3"/>
+          <min val="2"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>WAF</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="span"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>(나) 학습 상태 (0 = 전수 순회, 1 = 탐색, 2 = 정착)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <scatterStyle val="lineMarker"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'③ 마지막 30분 마지막 30분'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="2A78D6"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$E$2:$E$16</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$F$2:$F$16</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="10.05"/>
+          <min val="9.550000000000001"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>측정 시작 후 시간 (시간)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+        <majorUnit val="0.1"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="2.2"/>
+          <min val="-0.2"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>상태</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="span"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>(다) 활성 후보 수 (파티션 2)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <scatterStyle val="lineMarker"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'③ 마지막 30분 마지막 30분'!H1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="2A78D6"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$G$2:$G$16</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'③ 마지막 30분 마지막 30분'!$H$2:$H$16</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="10.05"/>
+          <min val="9.550000000000001"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -1109,6 +1564,77 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1468,7 +1994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1479,7 +2005,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>iCAT-v4 (제안) 10분 구간 WAF</t>
+          <t>iCAT-v4 (제안) 2분 구간 WAF</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1489,7 +2015,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>CAT-37 (기본값) 10분 구간 WAF</t>
+          <t>CAT-37 (기본값) 2분 구간 WAF</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1520,25 +2046,25 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.0833</v>
+        <v>0.0167</v>
       </c>
       <c r="B2" t="n">
-        <v>1.2837</v>
+        <v>1.3763</v>
       </c>
       <c r="C2" t="n">
         <v>0.0833</v>
       </c>
       <c r="D2" t="n">
-        <v>1.4671</v>
+        <v>1.5469</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0833</v>
+        <v>0.0167</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0833</v>
+        <v>0.0167</v>
       </c>
       <c r="H2" t="n">
         <v>45</v>
@@ -1549,28 +2075,28 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.25</v>
+        <v>0.05</v>
       </c>
       <c r="B3" t="n">
-        <v>1.2278</v>
+        <v>1.2722</v>
       </c>
       <c r="C3" t="n">
-        <v>0.25</v>
+        <v>0.1167</v>
       </c>
       <c r="D3" t="n">
-        <v>1.3935</v>
+        <v>1.4703</v>
       </c>
       <c r="E3" t="n">
-        <v>0.25</v>
+        <v>0.05</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.25</v>
+        <v>0.05</v>
       </c>
       <c r="H3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
@@ -1580,28 +2106,28 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.4167</v>
+        <v>0.0833</v>
       </c>
       <c r="B4" t="n">
-        <v>1.222</v>
+        <v>1.2803</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4167</v>
+        <v>0.15</v>
       </c>
       <c r="D4" t="n">
-        <v>1.3316</v>
+        <v>1.447</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4167</v>
+        <v>0.0833</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4167</v>
+        <v>0.0833</v>
       </c>
       <c r="H4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J4" t="n">
         <v>5.13</v>
@@ -1609,54 +2135,54 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.5833</v>
+        <v>0.1167</v>
       </c>
       <c r="B5" t="n">
-        <v>1.2219</v>
+        <v>1.2616</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5833</v>
+        <v>0.1833</v>
       </c>
       <c r="D5" t="n">
-        <v>1.3133</v>
+        <v>1.4239</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5833</v>
+        <v>0.1167</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5833</v>
+        <v>0.1167</v>
       </c>
       <c r="H5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.75</v>
+        <v>0.15</v>
       </c>
       <c r="B6" t="n">
-        <v>1.2208</v>
+        <v>1.2315</v>
       </c>
       <c r="C6" t="n">
-        <v>0.75</v>
+        <v>0.2167</v>
       </c>
       <c r="D6" t="n">
-        <v>1.3083</v>
+        <v>1.4095</v>
       </c>
       <c r="E6" t="n">
-        <v>0.75</v>
+        <v>0.15</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.75</v>
+        <v>0.15</v>
       </c>
       <c r="H6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1669,28 +2195,28 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.9167</v>
+        <v>0.1833</v>
       </c>
       <c r="B7" t="n">
-        <v>1.2158</v>
+        <v>1.2334</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9167</v>
+        <v>0.25</v>
       </c>
       <c r="D7" t="n">
-        <v>1.3034</v>
+        <v>1.3949</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9167</v>
+        <v>0.1833</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9167</v>
+        <v>0.1833</v>
       </c>
       <c r="H7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1703,77 +2229,77 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1.0833</v>
+        <v>0.2167</v>
       </c>
       <c r="B8" t="n">
-        <v>1.216</v>
+        <v>1.2304</v>
       </c>
       <c r="C8" t="n">
-        <v>1.0833</v>
+        <v>0.2833</v>
       </c>
       <c r="D8" t="n">
-        <v>1.2965</v>
+        <v>1.3764</v>
       </c>
       <c r="E8" t="n">
-        <v>1.0833</v>
+        <v>0.2167</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1.0833</v>
+        <v>0.2167</v>
       </c>
       <c r="H8" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1.25</v>
+        <v>0.25</v>
       </c>
       <c r="B9" t="n">
-        <v>1.2155</v>
+        <v>1.2243</v>
       </c>
       <c r="C9" t="n">
-        <v>1.25</v>
+        <v>0.3167</v>
       </c>
       <c r="D9" t="n">
-        <v>1.2904</v>
+        <v>1.3627</v>
       </c>
       <c r="E9" t="n">
-        <v>1.25</v>
+        <v>0.25</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1.25</v>
+        <v>0.25</v>
       </c>
       <c r="H9" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.4167</v>
+        <v>0.2833</v>
       </c>
       <c r="B10" t="n">
-        <v>1.2153</v>
+        <v>1.2251</v>
       </c>
       <c r="C10" t="n">
-        <v>1.4167</v>
+        <v>0.35</v>
       </c>
       <c r="D10" t="n">
-        <v>1.2912</v>
+        <v>1.3465</v>
       </c>
       <c r="E10" t="n">
-        <v>1.4167</v>
+        <v>0.2833</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1.4167</v>
+        <v>0.2833</v>
       </c>
       <c r="H10" t="n">
         <v>45</v>
@@ -1781,1328 +2307,536 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1.5833</v>
+        <v>0.3167</v>
       </c>
       <c r="B11" t="n">
-        <v>1.2188</v>
+        <v>1.2241</v>
       </c>
       <c r="C11" t="n">
-        <v>1.5833</v>
+        <v>0.3833</v>
       </c>
       <c r="D11" t="n">
-        <v>1.2887</v>
+        <v>1.3363</v>
       </c>
       <c r="E11" t="n">
-        <v>1.5833</v>
+        <v>0.3167</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1.5833</v>
+        <v>0.3167</v>
       </c>
       <c r="H11" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1.75</v>
+        <v>0.35</v>
       </c>
       <c r="B12" t="n">
-        <v>1.2222</v>
+        <v>1.2214</v>
       </c>
       <c r="C12" t="n">
-        <v>1.75</v>
+        <v>0.4167</v>
       </c>
       <c r="D12" t="n">
-        <v>1.2831</v>
+        <v>1.3286</v>
       </c>
       <c r="E12" t="n">
-        <v>1.75</v>
+        <v>0.35</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1.75</v>
+        <v>0.35</v>
       </c>
       <c r="H12" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1.9167</v>
+        <v>0.3833</v>
       </c>
       <c r="B13" t="n">
-        <v>1.2266</v>
+        <v>1.2232</v>
       </c>
       <c r="C13" t="n">
-        <v>1.9167</v>
+        <v>0.45</v>
       </c>
       <c r="D13" t="n">
-        <v>1.2872</v>
+        <v>1.3231</v>
       </c>
       <c r="E13" t="n">
-        <v>1.9167</v>
+        <v>0.3833</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>1.9167</v>
+        <v>0.3833</v>
       </c>
       <c r="H13" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2.0833</v>
+        <v>0.4167</v>
       </c>
       <c r="B14" t="n">
-        <v>1.226</v>
+        <v>1.2224</v>
       </c>
       <c r="C14" t="n">
-        <v>2.0833</v>
+        <v>0.4833</v>
       </c>
       <c r="D14" t="n">
-        <v>1.2874</v>
+        <v>1.3245</v>
       </c>
       <c r="E14" t="n">
-        <v>2.0833</v>
+        <v>0.4167</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>2.0833</v>
+        <v>0.4167</v>
       </c>
       <c r="H14" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2.25</v>
+        <v>0.45</v>
       </c>
       <c r="B15" t="n">
-        <v>1.2263</v>
+        <v>1.2219</v>
       </c>
       <c r="C15" t="n">
-        <v>2.25</v>
+        <v>0.5167</v>
       </c>
       <c r="D15" t="n">
-        <v>1.2859</v>
+        <v>1.3187</v>
       </c>
       <c r="E15" t="n">
-        <v>2.25</v>
+        <v>0.45</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>2.25</v>
+        <v>0.45</v>
       </c>
       <c r="H15" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2.4167</v>
+        <v>0.4833</v>
       </c>
       <c r="B16" t="n">
-        <v>1.2277</v>
+        <v>1.2208</v>
       </c>
       <c r="C16" t="n">
-        <v>2.4167</v>
+        <v>0.55</v>
       </c>
       <c r="D16" t="n">
-        <v>1.2862</v>
+        <v>1.3152</v>
       </c>
       <c r="E16" t="n">
-        <v>2.4167</v>
+        <v>0.4833</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>2.4167</v>
+        <v>0.4833</v>
       </c>
       <c r="H16" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2.5833</v>
+        <v>0.5167</v>
       </c>
       <c r="B17" t="n">
-        <v>1.2271</v>
+        <v>1.224</v>
       </c>
       <c r="C17" t="n">
-        <v>2.5833</v>
+        <v>0.5833</v>
       </c>
       <c r="D17" t="n">
-        <v>1.2858</v>
+        <v>1.3087</v>
       </c>
       <c r="E17" t="n">
-        <v>2.5833</v>
+        <v>0.5167</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>2.5833</v>
+        <v>0.5167</v>
       </c>
       <c r="H17" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2.75</v>
+        <v>0.55</v>
       </c>
       <c r="B18" t="n">
-        <v>1.227</v>
+        <v>1.2219</v>
       </c>
       <c r="C18" t="n">
-        <v>2.75</v>
+        <v>0.6167</v>
       </c>
       <c r="D18" t="n">
-        <v>1.283</v>
+        <v>1.3116</v>
       </c>
       <c r="E18" t="n">
-        <v>2.75</v>
+        <v>0.55</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>2.75</v>
+        <v>0.55</v>
       </c>
       <c r="H18" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2.9167</v>
+        <v>0.5833</v>
       </c>
       <c r="B19" t="n">
-        <v>1.2263</v>
+        <v>1.222</v>
       </c>
       <c r="C19" t="n">
-        <v>2.9167</v>
+        <v>0.65</v>
       </c>
       <c r="D19" t="n">
-        <v>1.2841</v>
+        <v>1.3123</v>
       </c>
       <c r="E19" t="n">
-        <v>2.9167</v>
+        <v>0.5833</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>2.9167</v>
+        <v>0.5833</v>
       </c>
       <c r="H19" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3.0833</v>
+        <v>0.6167</v>
       </c>
       <c r="B20" t="n">
-        <v>1.2224</v>
+        <v>1.221</v>
       </c>
       <c r="C20" t="n">
-        <v>3.0833</v>
+        <v>0.6833</v>
       </c>
       <c r="D20" t="n">
-        <v>1.2827</v>
+        <v>1.3099</v>
       </c>
       <c r="E20" t="n">
-        <v>3.0833</v>
+        <v>0.6167</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>3.0833</v>
+        <v>0.6167</v>
       </c>
       <c r="H20" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3.25</v>
+        <v>0.65</v>
       </c>
       <c r="B21" t="n">
-        <v>1.2244</v>
+        <v>1.2211</v>
       </c>
       <c r="C21" t="n">
-        <v>3.25</v>
+        <v>0.7167</v>
       </c>
       <c r="D21" t="n">
-        <v>1.2813</v>
+        <v>1.3083</v>
       </c>
       <c r="E21" t="n">
-        <v>3.25</v>
+        <v>0.65</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>3.25</v>
+        <v>0.65</v>
       </c>
       <c r="H21" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3.4167</v>
+        <v>0.6833</v>
       </c>
       <c r="B22" t="n">
-        <v>1.2274</v>
+        <v>1.2209</v>
       </c>
       <c r="C22" t="n">
-        <v>3.4167</v>
+        <v>0.75</v>
       </c>
       <c r="D22" t="n">
-        <v>1.282</v>
+        <v>1.3088</v>
       </c>
       <c r="E22" t="n">
-        <v>3.4167</v>
+        <v>0.6833</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>3.4167</v>
+        <v>0.6833</v>
       </c>
       <c r="H22" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3.5833</v>
+        <v>0.7167</v>
       </c>
       <c r="B23" t="n">
-        <v>1.2233</v>
+        <v>1.2219</v>
       </c>
       <c r="C23" t="n">
-        <v>3.5833</v>
+        <v>0.7833</v>
       </c>
       <c r="D23" t="n">
-        <v>1.2815</v>
+        <v>1.3072</v>
       </c>
       <c r="E23" t="n">
-        <v>3.5833</v>
+        <v>0.7167</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>3.5833</v>
+        <v>0.7167</v>
       </c>
       <c r="H23" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3.75</v>
+        <v>0.75</v>
       </c>
       <c r="B24" t="n">
-        <v>1.2242</v>
+        <v>1.2241</v>
       </c>
       <c r="C24" t="n">
-        <v>3.75</v>
+        <v>0.8167</v>
       </c>
       <c r="D24" t="n">
-        <v>1.2798</v>
+        <v>1.3072</v>
       </c>
       <c r="E24" t="n">
-        <v>3.75</v>
+        <v>0.75</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>3.75</v>
+        <v>0.75</v>
       </c>
       <c r="H24" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3.9167</v>
+        <v>0.7833</v>
       </c>
       <c r="B25" t="n">
-        <v>1.2276</v>
+        <v>1.2163</v>
       </c>
       <c r="C25" t="n">
-        <v>3.9167</v>
+        <v>0.85</v>
       </c>
       <c r="D25" t="n">
-        <v>1.2794</v>
+        <v>1.3055</v>
       </c>
       <c r="E25" t="n">
-        <v>3.9167</v>
+        <v>0.7833</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>3.9167</v>
+        <v>0.7833</v>
       </c>
       <c r="H25" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4.0833</v>
+        <v>0.8167</v>
       </c>
       <c r="B26" t="n">
-        <v>1.2251</v>
+        <v>1.2212</v>
       </c>
       <c r="C26" t="n">
-        <v>4.0833</v>
+        <v>0.8833</v>
       </c>
       <c r="D26" t="n">
-        <v>1.2788</v>
+        <v>1.3039</v>
       </c>
       <c r="E26" t="n">
-        <v>4.0833</v>
+        <v>0.8167</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>4.0833</v>
+        <v>0.8167</v>
       </c>
       <c r="H26" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>4.25</v>
+        <v>0.85</v>
       </c>
       <c r="B27" t="n">
-        <v>1.2229</v>
+        <v>1.2172</v>
       </c>
       <c r="C27" t="n">
-        <v>4.25</v>
+        <v>0.9167</v>
       </c>
       <c r="D27" t="n">
-        <v>1.2794</v>
+        <v>1.3021</v>
       </c>
       <c r="E27" t="n">
-        <v>4.25</v>
+        <v>0.85</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>4.25</v>
+        <v>0.85</v>
       </c>
       <c r="H27" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>4.4167</v>
+        <v>0.8833</v>
       </c>
       <c r="B28" t="n">
-        <v>1.2228</v>
+        <v>1.2156</v>
       </c>
       <c r="C28" t="n">
-        <v>4.4167</v>
+        <v>0.95</v>
       </c>
       <c r="D28" t="n">
-        <v>1.2841</v>
+        <v>1.3031</v>
       </c>
       <c r="E28" t="n">
-        <v>4.4167</v>
+        <v>0.8833</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>4.4167</v>
+        <v>0.8833</v>
       </c>
       <c r="H28" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>4.5833</v>
+        <v>0.9167</v>
       </c>
       <c r="B29" t="n">
-        <v>1.2198</v>
+        <v>1.2166</v>
       </c>
       <c r="C29" t="n">
-        <v>4.5833</v>
+        <v>0.9833</v>
       </c>
       <c r="D29" t="n">
-        <v>1.2811</v>
+        <v>1.3026</v>
       </c>
       <c r="E29" t="n">
-        <v>4.5833</v>
+        <v>0.9167</v>
       </c>
       <c r="F29" t="n">
         <v>2</v>
       </c>
       <c r="G29" t="n">
-        <v>4.5833</v>
+        <v>0.9167</v>
       </c>
       <c r="H29" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4.75</v>
+        <v>0.95</v>
       </c>
       <c r="B30" t="n">
-        <v>1.2178</v>
-      </c>
-      <c r="C30" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="D30" t="n">
-        <v>1.2815</v>
+        <v>1.2143</v>
       </c>
       <c r="E30" t="n">
-        <v>4.75</v>
+        <v>0.95</v>
       </c>
       <c r="F30" t="n">
         <v>2</v>
       </c>
       <c r="G30" t="n">
-        <v>4.75</v>
+        <v>0.95</v>
       </c>
       <c r="H30" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4.9167</v>
+        <v>0.9833</v>
       </c>
       <c r="B31" t="n">
-        <v>1.2264</v>
-      </c>
-      <c r="C31" t="n">
-        <v>4.9167</v>
-      </c>
-      <c r="D31" t="n">
-        <v>1.2832</v>
+        <v>1.2151</v>
       </c>
       <c r="E31" t="n">
-        <v>4.9167</v>
+        <v>0.9833</v>
       </c>
       <c r="F31" t="n">
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>4.9167</v>
+        <v>0.9833</v>
       </c>
       <c r="H31" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>5.0833</v>
-      </c>
-      <c r="B32" t="n">
-        <v>2.0097</v>
-      </c>
-      <c r="C32" t="n">
-        <v>5.0833</v>
-      </c>
-      <c r="D32" t="n">
-        <v>1.9526</v>
-      </c>
-      <c r="E32" t="n">
-        <v>5.0833</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" t="n">
-        <v>5.0833</v>
-      </c>
-      <c r="H32" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="B33" t="n">
-        <v>2.0751</v>
-      </c>
-      <c r="C33" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="D33" t="n">
-        <v>2.4273</v>
-      </c>
-      <c r="E33" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="F33" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="H33" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>5.4167</v>
-      </c>
-      <c r="B34" t="n">
-        <v>2.0654</v>
-      </c>
-      <c r="C34" t="n">
-        <v>5.4167</v>
-      </c>
-      <c r="D34" t="n">
-        <v>2.4194</v>
-      </c>
-      <c r="E34" t="n">
-        <v>5.4167</v>
-      </c>
-      <c r="F34" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" t="n">
-        <v>5.4167</v>
-      </c>
-      <c r="H34" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>5.5833</v>
-      </c>
-      <c r="B35" t="n">
-        <v>2.0594</v>
-      </c>
-      <c r="C35" t="n">
-        <v>5.5833</v>
-      </c>
-      <c r="D35" t="n">
-        <v>2.4076</v>
-      </c>
-      <c r="E35" t="n">
-        <v>5.5833</v>
-      </c>
-      <c r="F35" t="n">
-        <v>2</v>
-      </c>
-      <c r="G35" t="n">
-        <v>5.5833</v>
-      </c>
-      <c r="H35" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="B36" t="n">
-        <v>2.0601</v>
-      </c>
-      <c r="C36" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="D36" t="n">
-        <v>2.3992</v>
-      </c>
-      <c r="E36" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="F36" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="H36" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>5.9167</v>
-      </c>
-      <c r="B37" t="n">
-        <v>2.054</v>
-      </c>
-      <c r="C37" t="n">
-        <v>5.9167</v>
-      </c>
-      <c r="D37" t="n">
-        <v>2.388</v>
-      </c>
-      <c r="E37" t="n">
-        <v>5.9167</v>
-      </c>
-      <c r="F37" t="n">
-        <v>2</v>
-      </c>
-      <c r="G37" t="n">
-        <v>5.9167</v>
-      </c>
-      <c r="H37" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>6.0833</v>
-      </c>
-      <c r="B38" t="n">
-        <v>2.0545</v>
-      </c>
-      <c r="C38" t="n">
-        <v>6.0833</v>
-      </c>
-      <c r="D38" t="n">
-        <v>2.3808</v>
-      </c>
-      <c r="E38" t="n">
-        <v>6.0833</v>
-      </c>
-      <c r="F38" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" t="n">
-        <v>6.0833</v>
-      </c>
-      <c r="H38" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="B39" t="n">
-        <v>2.0534</v>
-      </c>
-      <c r="C39" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="D39" t="n">
-        <v>2.3726</v>
-      </c>
-      <c r="E39" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="F39" t="n">
-        <v>2</v>
-      </c>
-      <c r="G39" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="H39" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>6.4167</v>
-      </c>
-      <c r="B40" t="n">
-        <v>2.0528</v>
-      </c>
-      <c r="C40" t="n">
-        <v>6.4167</v>
-      </c>
-      <c r="D40" t="n">
-        <v>2.365</v>
-      </c>
-      <c r="E40" t="n">
-        <v>6.4167</v>
-      </c>
-      <c r="F40" t="n">
-        <v>2</v>
-      </c>
-      <c r="G40" t="n">
-        <v>6.4167</v>
-      </c>
-      <c r="H40" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>6.5833</v>
-      </c>
-      <c r="B41" t="n">
-        <v>2.0522</v>
-      </c>
-      <c r="C41" t="n">
-        <v>6.5833</v>
-      </c>
-      <c r="D41" t="n">
-        <v>2.3586</v>
-      </c>
-      <c r="E41" t="n">
-        <v>6.5833</v>
-      </c>
-      <c r="F41" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" t="n">
-        <v>6.5833</v>
-      </c>
-      <c r="H41" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="B42" t="n">
-        <v>2.0526</v>
-      </c>
-      <c r="C42" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="D42" t="n">
-        <v>2.3521</v>
-      </c>
-      <c r="E42" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="F42" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="H42" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>6.9167</v>
-      </c>
-      <c r="B43" t="n">
-        <v>2.0521</v>
-      </c>
-      <c r="C43" t="n">
-        <v>6.9167</v>
-      </c>
-      <c r="D43" t="n">
-        <v>2.3454</v>
-      </c>
-      <c r="E43" t="n">
-        <v>6.9167</v>
-      </c>
-      <c r="F43" t="n">
-        <v>2</v>
-      </c>
-      <c r="G43" t="n">
-        <v>6.9167</v>
-      </c>
-      <c r="H43" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>7.0833</v>
-      </c>
-      <c r="B44" t="n">
-        <v>2.0512</v>
-      </c>
-      <c r="C44" t="n">
-        <v>7.0833</v>
-      </c>
-      <c r="D44" t="n">
-        <v>2.3403</v>
-      </c>
-      <c r="E44" t="n">
-        <v>7.0833</v>
-      </c>
-      <c r="F44" t="n">
-        <v>2</v>
-      </c>
-      <c r="G44" t="n">
-        <v>7.0833</v>
-      </c>
-      <c r="H44" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="B45" t="n">
-        <v>2.0507</v>
-      </c>
-      <c r="C45" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="D45" t="n">
-        <v>2.3347</v>
-      </c>
-      <c r="E45" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="F45" t="n">
-        <v>2</v>
-      </c>
-      <c r="G45" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="H45" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>7.4167</v>
-      </c>
-      <c r="B46" t="n">
-        <v>2.0507</v>
-      </c>
-      <c r="C46" t="n">
-        <v>7.4167</v>
-      </c>
-      <c r="D46" t="n">
-        <v>2.3301</v>
-      </c>
-      <c r="E46" t="n">
-        <v>7.4167</v>
-      </c>
-      <c r="F46" t="n">
-        <v>2</v>
-      </c>
-      <c r="G46" t="n">
-        <v>7.4167</v>
-      </c>
-      <c r="H46" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>7.5833</v>
-      </c>
-      <c r="B47" t="n">
-        <v>2.0484</v>
-      </c>
-      <c r="C47" t="n">
-        <v>7.5833</v>
-      </c>
-      <c r="D47" t="n">
-        <v>2.3267</v>
-      </c>
-      <c r="E47" t="n">
-        <v>7.5833</v>
-      </c>
-      <c r="F47" t="n">
-        <v>2</v>
-      </c>
-      <c r="G47" t="n">
-        <v>7.5833</v>
-      </c>
-      <c r="H47" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="B48" t="n">
-        <v>2.0493</v>
-      </c>
-      <c r="C48" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="D48" t="n">
-        <v>2.3209</v>
-      </c>
-      <c r="E48" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="F48" t="n">
-        <v>2</v>
-      </c>
-      <c r="G48" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="H48" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>7.9167</v>
-      </c>
-      <c r="B49" t="n">
-        <v>2.048</v>
-      </c>
-      <c r="C49" t="n">
-        <v>7.9167</v>
-      </c>
-      <c r="D49" t="n">
-        <v>2.3172</v>
-      </c>
-      <c r="E49" t="n">
-        <v>7.9167</v>
-      </c>
-      <c r="F49" t="n">
-        <v>2</v>
-      </c>
-      <c r="G49" t="n">
-        <v>7.9167</v>
-      </c>
-      <c r="H49" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>8.083299999999999</v>
-      </c>
-      <c r="B50" t="n">
-        <v>2.0479</v>
-      </c>
-      <c r="C50" t="n">
-        <v>8.083299999999999</v>
-      </c>
-      <c r="D50" t="n">
-        <v>2.3139</v>
-      </c>
-      <c r="E50" t="n">
-        <v>8.083299999999999</v>
-      </c>
-      <c r="F50" t="n">
-        <v>2</v>
-      </c>
-      <c r="G50" t="n">
-        <v>8.083299999999999</v>
-      </c>
-      <c r="H50" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="B51" t="n">
-        <v>2.0475</v>
-      </c>
-      <c r="C51" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="D51" t="n">
-        <v>2.311</v>
-      </c>
-      <c r="E51" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="F51" t="n">
-        <v>2</v>
-      </c>
-      <c r="G51" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="H51" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>8.416700000000001</v>
-      </c>
-      <c r="B52" t="n">
-        <v>2.0475</v>
-      </c>
-      <c r="C52" t="n">
-        <v>8.416700000000001</v>
-      </c>
-      <c r="D52" t="n">
-        <v>2.3076</v>
-      </c>
-      <c r="E52" t="n">
-        <v>8.416700000000001</v>
-      </c>
-      <c r="F52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G52" t="n">
-        <v>8.416700000000001</v>
-      </c>
-      <c r="H52" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>8.583299999999999</v>
-      </c>
-      <c r="B53" t="n">
-        <v>2.0458</v>
-      </c>
-      <c r="C53" t="n">
-        <v>8.583299999999999</v>
-      </c>
-      <c r="D53" t="n">
-        <v>2.3056</v>
-      </c>
-      <c r="E53" t="n">
-        <v>8.583299999999999</v>
-      </c>
-      <c r="F53" t="n">
-        <v>2</v>
-      </c>
-      <c r="G53" t="n">
-        <v>8.583299999999999</v>
-      </c>
-      <c r="H53" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="B54" t="n">
-        <v>2.0471</v>
-      </c>
-      <c r="C54" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="D54" t="n">
-        <v>2.3024</v>
-      </c>
-      <c r="E54" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="F54" t="n">
-        <v>2</v>
-      </c>
-      <c r="G54" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="H54" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>8.916700000000001</v>
-      </c>
-      <c r="B55" t="n">
-        <v>2.0462</v>
-      </c>
-      <c r="C55" t="n">
-        <v>8.916700000000001</v>
-      </c>
-      <c r="D55" t="n">
-        <v>2.299</v>
-      </c>
-      <c r="E55" t="n">
-        <v>8.916700000000001</v>
-      </c>
-      <c r="F55" t="n">
-        <v>2</v>
-      </c>
-      <c r="G55" t="n">
-        <v>8.916700000000001</v>
-      </c>
-      <c r="H55" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>9.083299999999999</v>
-      </c>
-      <c r="B56" t="n">
-        <v>2.0471</v>
-      </c>
-      <c r="C56" t="n">
-        <v>9.083299999999999</v>
-      </c>
-      <c r="D56" t="n">
-        <v>2.297</v>
-      </c>
-      <c r="E56" t="n">
-        <v>9.083299999999999</v>
-      </c>
-      <c r="F56" t="n">
-        <v>2</v>
-      </c>
-      <c r="G56" t="n">
-        <v>9.083299999999999</v>
-      </c>
-      <c r="H56" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="B57" t="n">
-        <v>2.0455</v>
-      </c>
-      <c r="C57" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="D57" t="n">
-        <v>2.2957</v>
-      </c>
-      <c r="E57" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="F57" t="n">
-        <v>2</v>
-      </c>
-      <c r="G57" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="H57" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>9.416700000000001</v>
-      </c>
-      <c r="B58" t="n">
-        <v>2.046</v>
-      </c>
-      <c r="C58" t="n">
-        <v>9.416700000000001</v>
-      </c>
-      <c r="D58" t="n">
-        <v>2.2938</v>
-      </c>
-      <c r="E58" t="n">
-        <v>9.416700000000001</v>
-      </c>
-      <c r="F58" t="n">
-        <v>2</v>
-      </c>
-      <c r="G58" t="n">
-        <v>9.416700000000001</v>
-      </c>
-      <c r="H58" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>9.583299999999999</v>
-      </c>
-      <c r="B59" t="n">
-        <v>2.0455</v>
-      </c>
-      <c r="C59" t="n">
-        <v>9.583299999999999</v>
-      </c>
-      <c r="D59" t="n">
-        <v>2.2919</v>
-      </c>
-      <c r="E59" t="n">
-        <v>9.583299999999999</v>
-      </c>
-      <c r="F59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G59" t="n">
-        <v>9.583299999999999</v>
-      </c>
-      <c r="H59" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="B60" t="n">
-        <v>2.0454</v>
-      </c>
-      <c r="C60" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="D60" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="E60" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="F60" t="n">
-        <v>2</v>
-      </c>
-      <c r="G60" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="H60" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>9.916700000000001</v>
-      </c>
-      <c r="B61" t="n">
-        <v>2.0452</v>
-      </c>
-      <c r="C61" t="n">
-        <v>9.916700000000001</v>
-      </c>
-      <c r="D61" t="n">
-        <v>2.2871</v>
-      </c>
-      <c r="E61" t="n">
-        <v>9.916700000000001</v>
-      </c>
-      <c r="F61" t="n">
-        <v>2</v>
-      </c>
-      <c r="G61" t="n">
-        <v>9.916700000000001</v>
-      </c>
-      <c r="H61" t="n">
-        <v>12</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -3117,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3128,7 +2862,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>iCAT-v4 (제안) 1분 구간 WAF</t>
+          <t>iCAT-v4 (제안) 2분 구간 WAF</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3138,7 +2872,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>CAT-37 (기본값) 1분 구간 WAF</t>
+          <t>CAT-37 (기본값) 2분 구간 WAF</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -3169,25 +2903,25 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4.9572</v>
+        <v>4.9656</v>
       </c>
       <c r="B2" t="n">
         <v>1.227</v>
       </c>
       <c r="C2" t="n">
-        <v>4.9572</v>
+        <v>4.9656</v>
       </c>
       <c r="D2" t="n">
-        <v>1.2841</v>
+        <v>1.2839</v>
       </c>
       <c r="E2" t="n">
-        <v>4.9572</v>
+        <v>4.9656</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>4.9572</v>
+        <v>4.9656</v>
       </c>
       <c r="H2" t="n">
         <v>45</v>
@@ -3198,25 +2932,25 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4.9739</v>
+        <v>4.9989</v>
       </c>
       <c r="B3" t="n">
-        <v>1.227</v>
+        <v>1.2264</v>
       </c>
       <c r="C3" t="n">
-        <v>4.9739</v>
+        <v>4.9989</v>
       </c>
       <c r="D3" t="n">
-        <v>1.2838</v>
+        <v>1.2816</v>
       </c>
       <c r="E3" t="n">
-        <v>4.9739</v>
+        <v>4.9989</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>4.9739</v>
+        <v>4.9989</v>
       </c>
       <c r="H3" t="n">
         <v>45</v>
@@ -3229,25 +2963,25 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4.9906</v>
+        <v>5.0322</v>
       </c>
       <c r="B4" t="n">
-        <v>1.2271</v>
+        <v>1.2263</v>
       </c>
       <c r="C4" t="n">
-        <v>4.9906</v>
+        <v>5.0322</v>
       </c>
       <c r="D4" t="n">
-        <v>1.2822</v>
+        <v>1.2805</v>
       </c>
       <c r="E4" t="n">
-        <v>4.9906</v>
+        <v>5.0322</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>4.9906</v>
+        <v>5.0322</v>
       </c>
       <c r="H4" t="n">
         <v>45</v>
@@ -3258,54 +2992,54 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5.0072</v>
+        <v>5.0656</v>
       </c>
       <c r="B5" t="n">
-        <v>1.2256</v>
+        <v>2.0441</v>
       </c>
       <c r="C5" t="n">
-        <v>5.0072</v>
+        <v>5.0656</v>
       </c>
       <c r="D5" t="n">
-        <v>1.281</v>
+        <v>1.2815</v>
       </c>
       <c r="E5" t="n">
-        <v>5.0072</v>
+        <v>5.0656</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>5.0072</v>
+        <v>5.0656</v>
       </c>
       <c r="H5" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5.0239</v>
+        <v>5.0989</v>
       </c>
       <c r="B6" t="n">
-        <v>1.2265</v>
+        <v>2.0819</v>
       </c>
       <c r="C6" t="n">
-        <v>5.0239</v>
+        <v>5.0989</v>
       </c>
       <c r="D6" t="n">
-        <v>1.2822</v>
+        <v>1.2852</v>
       </c>
       <c r="E6" t="n">
-        <v>5.0239</v>
+        <v>5.0989</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>5.0239</v>
+        <v>5.0989</v>
       </c>
       <c r="H6" t="n">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -3318,28 +3052,28 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5.0406</v>
+        <v>5.1322</v>
       </c>
       <c r="B7" t="n">
-        <v>1.2262</v>
+        <v>2.0839</v>
       </c>
       <c r="C7" t="n">
-        <v>5.0406</v>
+        <v>5.1322</v>
       </c>
       <c r="D7" t="n">
-        <v>1.2787</v>
+        <v>2.342</v>
       </c>
       <c r="E7" t="n">
-        <v>5.0406</v>
+        <v>5.1322</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>5.0406</v>
+        <v>5.1322</v>
       </c>
       <c r="H7" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -3352,259 +3086,259 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>5.0572</v>
+        <v>5.1656</v>
       </c>
       <c r="B8" t="n">
-        <v>1.9892</v>
+        <v>2.0852</v>
       </c>
       <c r="C8" t="n">
-        <v>5.0572</v>
+        <v>5.1656</v>
       </c>
       <c r="D8" t="n">
-        <v>1.2818</v>
+        <v>2.4259</v>
       </c>
       <c r="E8" t="n">
-        <v>5.0572</v>
+        <v>5.1656</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>5.0572</v>
+        <v>5.1656</v>
       </c>
       <c r="H8" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>5.0739</v>
+        <v>5.1989</v>
       </c>
       <c r="B9" t="n">
-        <v>2.0915</v>
+        <v>2.0764</v>
       </c>
       <c r="C9" t="n">
-        <v>5.0739</v>
+        <v>5.1989</v>
       </c>
       <c r="D9" t="n">
-        <v>1.2812</v>
+        <v>2.428</v>
       </c>
       <c r="E9" t="n">
-        <v>5.0739</v>
+        <v>5.1989</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>5.0739</v>
+        <v>5.1989</v>
       </c>
       <c r="H9" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5.0906</v>
+        <v>5.2322</v>
       </c>
       <c r="B10" t="n">
-        <v>2.0814</v>
+        <v>2.0724</v>
       </c>
       <c r="C10" t="n">
-        <v>5.0906</v>
+        <v>5.2322</v>
       </c>
       <c r="D10" t="n">
-        <v>1.2823</v>
+        <v>2.4276</v>
       </c>
       <c r="E10" t="n">
-        <v>5.0906</v>
+        <v>5.2322</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>5.0906</v>
+        <v>5.2322</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5.1072</v>
+        <v>5.2656</v>
       </c>
       <c r="B11" t="n">
-        <v>2.0823</v>
+        <v>2.0722</v>
       </c>
       <c r="C11" t="n">
-        <v>5.1072</v>
+        <v>5.2656</v>
       </c>
       <c r="D11" t="n">
-        <v>1.288</v>
+        <v>2.4287</v>
       </c>
       <c r="E11" t="n">
-        <v>5.1072</v>
+        <v>5.2656</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>5.1072</v>
+        <v>5.2656</v>
       </c>
       <c r="H11" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>5.1239</v>
+        <v>5.2989</v>
       </c>
       <c r="B12" t="n">
-        <v>2.0851</v>
+        <v>2.0748</v>
       </c>
       <c r="C12" t="n">
-        <v>5.1239</v>
+        <v>5.2989</v>
       </c>
       <c r="D12" t="n">
-        <v>2.265</v>
+        <v>2.4263</v>
       </c>
       <c r="E12" t="n">
-        <v>5.1239</v>
+        <v>5.2989</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>5.1239</v>
+        <v>5.2989</v>
       </c>
       <c r="H12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5.1406</v>
+        <v>5.3322</v>
       </c>
       <c r="B13" t="n">
-        <v>2.0827</v>
+        <v>2.0727</v>
       </c>
       <c r="C13" t="n">
-        <v>5.1406</v>
+        <v>5.3322</v>
       </c>
       <c r="D13" t="n">
-        <v>2.4196</v>
+        <v>2.4228</v>
       </c>
       <c r="E13" t="n">
-        <v>5.1406</v>
+        <v>5.3322</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>5.1406</v>
+        <v>5.3322</v>
       </c>
       <c r="H13" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>5.1572</v>
+        <v>5.3656</v>
       </c>
       <c r="B14" t="n">
-        <v>2.0845</v>
+        <v>2.072</v>
       </c>
       <c r="C14" t="n">
-        <v>5.1572</v>
+        <v>5.3656</v>
       </c>
       <c r="D14" t="n">
-        <v>2.4242</v>
+        <v>2.4221</v>
       </c>
       <c r="E14" t="n">
-        <v>5.1572</v>
+        <v>5.3656</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>5.1572</v>
+        <v>5.3656</v>
       </c>
       <c r="H14" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5.1739</v>
+        <v>5.3989</v>
       </c>
       <c r="B15" t="n">
-        <v>2.0859</v>
+        <v>2.0679</v>
       </c>
       <c r="C15" t="n">
-        <v>5.1739</v>
+        <v>5.3989</v>
       </c>
       <c r="D15" t="n">
-        <v>2.4276</v>
+        <v>2.4225</v>
       </c>
       <c r="E15" t="n">
-        <v>5.1739</v>
+        <v>5.3989</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>5.1739</v>
+        <v>5.3989</v>
       </c>
       <c r="H15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5.1906</v>
+        <v>5.4322</v>
       </c>
       <c r="B16" t="n">
-        <v>2.0782</v>
+        <v>2.0594</v>
       </c>
       <c r="C16" t="n">
-        <v>5.1906</v>
+        <v>5.4322</v>
       </c>
       <c r="D16" t="n">
-        <v>2.4308</v>
+        <v>2.4205</v>
       </c>
       <c r="E16" t="n">
-        <v>5.1906</v>
+        <v>5.4322</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>5.1906</v>
+        <v>5.4322</v>
       </c>
       <c r="H16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>5.2072</v>
+        <v>5.4656</v>
       </c>
       <c r="B17" t="n">
-        <v>2.0745</v>
+        <v>2.0609</v>
       </c>
       <c r="C17" t="n">
-        <v>5.2072</v>
+        <v>5.4656</v>
       </c>
       <c r="D17" t="n">
-        <v>2.4251</v>
+        <v>2.415</v>
       </c>
       <c r="E17" t="n">
-        <v>5.2072</v>
+        <v>5.4656</v>
       </c>
       <c r="F17" t="n">
         <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>5.2072</v>
+        <v>5.4656</v>
       </c>
       <c r="H17" t="n">
         <v>12</v>
@@ -3612,25 +3346,25 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5.2239</v>
+        <v>5.4989</v>
       </c>
       <c r="B18" t="n">
-        <v>2.0718</v>
+        <v>2.0612</v>
       </c>
       <c r="C18" t="n">
-        <v>5.2239</v>
+        <v>5.4989</v>
       </c>
       <c r="D18" t="n">
-        <v>2.4273</v>
+        <v>2.4122</v>
       </c>
       <c r="E18" t="n">
-        <v>5.2239</v>
+        <v>5.4989</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>5.2239</v>
+        <v>5.4989</v>
       </c>
       <c r="H18" t="n">
         <v>12</v>
@@ -3638,25 +3372,25 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>5.2406</v>
+        <v>5.5322</v>
       </c>
       <c r="B19" t="n">
-        <v>2.073</v>
+        <v>2.0562</v>
       </c>
       <c r="C19" t="n">
-        <v>5.2406</v>
+        <v>5.5322</v>
       </c>
       <c r="D19" t="n">
-        <v>2.4278</v>
+        <v>2.4083</v>
       </c>
       <c r="E19" t="n">
-        <v>5.2406</v>
+        <v>5.5322</v>
       </c>
       <c r="F19" t="n">
         <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>5.2406</v>
+        <v>5.5322</v>
       </c>
       <c r="H19" t="n">
         <v>12</v>
@@ -3664,25 +3398,25 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>5.2572</v>
+        <v>5.5656</v>
       </c>
       <c r="B20" t="n">
-        <v>2.073</v>
+        <v>2.0596</v>
       </c>
       <c r="C20" t="n">
-        <v>5.2572</v>
+        <v>5.5656</v>
       </c>
       <c r="D20" t="n">
-        <v>2.4304</v>
+        <v>2.4076</v>
       </c>
       <c r="E20" t="n">
-        <v>5.2572</v>
+        <v>5.5656</v>
       </c>
       <c r="F20" t="n">
         <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>5.2572</v>
+        <v>5.5656</v>
       </c>
       <c r="H20" t="n">
         <v>12</v>
@@ -3690,25 +3424,25 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>5.2739</v>
+        <v>5.5989</v>
       </c>
       <c r="B21" t="n">
-        <v>2.0714</v>
+        <v>2.0599</v>
       </c>
       <c r="C21" t="n">
-        <v>5.2739</v>
+        <v>5.5989</v>
       </c>
       <c r="D21" t="n">
-        <v>2.427</v>
+        <v>2.4083</v>
       </c>
       <c r="E21" t="n">
-        <v>5.2739</v>
+        <v>5.5989</v>
       </c>
       <c r="F21" t="n">
         <v>2</v>
       </c>
       <c r="G21" t="n">
-        <v>5.2739</v>
+        <v>5.5989</v>
       </c>
       <c r="H21" t="n">
         <v>12</v>
@@ -3716,25 +3450,25 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>5.2906</v>
+        <v>5.6322</v>
       </c>
       <c r="B22" t="n">
-        <v>2.0758</v>
+        <v>2.061</v>
       </c>
       <c r="C22" t="n">
-        <v>5.2906</v>
+        <v>5.6322</v>
       </c>
       <c r="D22" t="n">
-        <v>2.4262</v>
+        <v>2.4063</v>
       </c>
       <c r="E22" t="n">
-        <v>5.2906</v>
+        <v>5.6322</v>
       </c>
       <c r="F22" t="n">
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>5.2906</v>
+        <v>5.6322</v>
       </c>
       <c r="H22" t="n">
         <v>12</v>
@@ -3742,25 +3476,25 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>5.3072</v>
+        <v>5.6656</v>
       </c>
       <c r="B23" t="n">
-        <v>2.0739</v>
+        <v>2.0603</v>
       </c>
       <c r="C23" t="n">
-        <v>5.3072</v>
+        <v>5.6656</v>
       </c>
       <c r="D23" t="n">
-        <v>2.4264</v>
+        <v>2.4038</v>
       </c>
       <c r="E23" t="n">
-        <v>5.3072</v>
+        <v>5.6656</v>
       </c>
       <c r="F23" t="n">
         <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>5.3072</v>
+        <v>5.6656</v>
       </c>
       <c r="H23" t="n">
         <v>12</v>
@@ -3768,25 +3502,25 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>5.3239</v>
+        <v>5.6989</v>
       </c>
       <c r="B24" t="n">
-        <v>2.0733</v>
+        <v>2.0656</v>
       </c>
       <c r="C24" t="n">
-        <v>5.3239</v>
+        <v>5.6989</v>
       </c>
       <c r="D24" t="n">
-        <v>2.4238</v>
+        <v>2.4013</v>
       </c>
       <c r="E24" t="n">
-        <v>5.3239</v>
+        <v>5.6989</v>
       </c>
       <c r="F24" t="n">
         <v>2</v>
       </c>
       <c r="G24" t="n">
-        <v>5.3239</v>
+        <v>5.6989</v>
       </c>
       <c r="H24" t="n">
         <v>12</v>
@@ -3794,495 +3528,500 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>5.3406</v>
+        <v>5.7322</v>
       </c>
       <c r="B25" t="n">
-        <v>2.0721</v>
+        <v>2.0633</v>
       </c>
       <c r="C25" t="n">
-        <v>5.3406</v>
+        <v>5.7322</v>
       </c>
       <c r="D25" t="n">
-        <v>2.4218</v>
+        <v>2.4026</v>
       </c>
       <c r="E25" t="n">
-        <v>5.3406</v>
+        <v>5.7322</v>
       </c>
       <c r="F25" t="n">
         <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>5.3406</v>
+        <v>5.7322</v>
       </c>
       <c r="H25" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>5.3572</v>
-      </c>
-      <c r="B26" t="n">
-        <v>2.0725</v>
-      </c>
-      <c r="C26" t="n">
-        <v>5.3572</v>
-      </c>
-      <c r="D26" t="n">
-        <v>2.4218</v>
-      </c>
-      <c r="E26" t="n">
-        <v>5.3572</v>
-      </c>
-      <c r="F26" t="n">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>iCAT-v4 (제안) 시간(h)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>iCAT-v4 (제안) 2분 구간 WAF</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-37 (기본값) 시간(h)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-37 (기본값) 2분 구간 WAF</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>시간(h)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>학습 상태 p2 (0=순회,1=탐색,2=정착)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">시간(h) </t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>남은 후보 수 p2</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>전환(시간)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>9.568</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2.0458</v>
+      </c>
+      <c r="C2" t="n">
+        <v>9.568</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.2932</v>
+      </c>
+      <c r="E2" t="n">
+        <v>9.568</v>
+      </c>
+      <c r="F2" t="n">
         <v>2</v>
       </c>
-      <c r="G26" t="n">
-        <v>5.3572</v>
-      </c>
-      <c r="H26" t="n">
+      <c r="G2" t="n">
+        <v>9.568</v>
+      </c>
+      <c r="H2" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>5.3739</v>
-      </c>
-      <c r="B27" t="n">
-        <v>2.0715</v>
-      </c>
-      <c r="C27" t="n">
-        <v>5.3739</v>
-      </c>
-      <c r="D27" t="n">
-        <v>2.4225</v>
-      </c>
-      <c r="E27" t="n">
-        <v>5.3739</v>
-      </c>
-      <c r="F27" t="n">
+      <c r="J2" t="n">
+        <v>5.049</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>9.6013</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2.0457</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9.6013</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.2907</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9.6013</v>
+      </c>
+      <c r="F3" t="n">
         <v>2</v>
       </c>
-      <c r="G27" t="n">
-        <v>5.3739</v>
-      </c>
-      <c r="H27" t="n">
+      <c r="G3" t="n">
+        <v>9.6013</v>
+      </c>
+      <c r="H3" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>5.3906</v>
-      </c>
-      <c r="B28" t="n">
-        <v>2.0706</v>
-      </c>
-      <c r="C28" t="n">
-        <v>5.3906</v>
-      </c>
-      <c r="D28" t="n">
-        <v>2.4231</v>
-      </c>
-      <c r="E28" t="n">
-        <v>5.3906</v>
-      </c>
-      <c r="F28" t="n">
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>재설정(시간, p2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>9.6347</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2.0466</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9.6347</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.2924</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9.6347</v>
+      </c>
+      <c r="F4" t="n">
         <v>2</v>
       </c>
-      <c r="G28" t="n">
-        <v>5.3906</v>
-      </c>
-      <c r="H28" t="n">
+      <c r="G4" t="n">
+        <v>9.6347</v>
+      </c>
+      <c r="H4" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>5.4072</v>
-      </c>
-      <c r="B29" t="n">
-        <v>2.0652</v>
-      </c>
-      <c r="C29" t="n">
-        <v>5.4072</v>
-      </c>
-      <c r="D29" t="n">
-        <v>2.4219</v>
-      </c>
-      <c r="E29" t="n">
-        <v>5.4072</v>
-      </c>
-      <c r="F29" t="n">
+      <c r="J4" t="n">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>9.667999999999999</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2.0452</v>
+      </c>
+      <c r="C5" t="n">
+        <v>9.667999999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.2915</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9.667999999999999</v>
+      </c>
+      <c r="F5" t="n">
         <v>2</v>
       </c>
-      <c r="G29" t="n">
-        <v>5.4072</v>
-      </c>
-      <c r="H29" t="n">
+      <c r="G5" t="n">
+        <v>9.667999999999999</v>
+      </c>
+      <c r="H5" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>5.4239</v>
-      </c>
-      <c r="B30" t="n">
-        <v>2.0603</v>
-      </c>
-      <c r="C30" t="n">
-        <v>5.4239</v>
-      </c>
-      <c r="D30" t="n">
-        <v>2.4229</v>
-      </c>
-      <c r="E30" t="n">
-        <v>5.4239</v>
-      </c>
-      <c r="F30" t="n">
+    <row r="6">
+      <c r="A6" t="n">
+        <v>9.7013</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2.0466</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9.7013</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.2914</v>
+      </c>
+      <c r="E6" t="n">
+        <v>9.7013</v>
+      </c>
+      <c r="F6" t="n">
         <v>2</v>
       </c>
-      <c r="G30" t="n">
-        <v>5.4239</v>
-      </c>
-      <c r="H30" t="n">
+      <c r="G6" t="n">
+        <v>9.7013</v>
+      </c>
+      <c r="H6" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>5.4406</v>
-      </c>
-      <c r="B31" t="n">
-        <v>2.0586</v>
-      </c>
-      <c r="C31" t="n">
-        <v>5.4406</v>
-      </c>
-      <c r="D31" t="n">
-        <v>2.4181</v>
-      </c>
-      <c r="E31" t="n">
-        <v>5.4406</v>
-      </c>
-      <c r="F31" t="n">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>iCAT-v4 (제안) 10시간 전체 WAF</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1.927</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>9.7347</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2.0458</v>
+      </c>
+      <c r="C7" t="n">
+        <v>9.7347</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.2906</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9.7347</v>
+      </c>
+      <c r="F7" t="n">
         <v>2</v>
       </c>
-      <c r="G31" t="n">
-        <v>5.4406</v>
-      </c>
-      <c r="H31" t="n">
+      <c r="G7" t="n">
+        <v>9.7347</v>
+      </c>
+      <c r="H7" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>5.4572</v>
-      </c>
-      <c r="B32" t="n">
-        <v>2.0609</v>
-      </c>
-      <c r="C32" t="n">
-        <v>5.4572</v>
-      </c>
-      <c r="D32" t="n">
-        <v>2.4165</v>
-      </c>
-      <c r="E32" t="n">
-        <v>5.4572</v>
-      </c>
-      <c r="F32" t="n">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>CAT-37 (기본값) 10시간 전체 WAF</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>2.122</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9.768000000000001</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2.045</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9.768000000000001</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.2894</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9.768000000000001</v>
+      </c>
+      <c r="F8" t="n">
         <v>2</v>
       </c>
-      <c r="G32" t="n">
-        <v>5.4572</v>
-      </c>
-      <c r="H32" t="n">
+      <c r="G8" t="n">
+        <v>9.768000000000001</v>
+      </c>
+      <c r="H8" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>5.4739</v>
-      </c>
-      <c r="B33" t="n">
-        <v>2.0609</v>
-      </c>
-      <c r="C33" t="n">
-        <v>5.4739</v>
-      </c>
-      <c r="D33" t="n">
-        <v>2.4136</v>
-      </c>
-      <c r="E33" t="n">
-        <v>5.4739</v>
-      </c>
-      <c r="F33" t="n">
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9.801299999999999</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2.0434</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9.801299999999999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.2884</v>
+      </c>
+      <c r="E9" t="n">
+        <v>9.801299999999999</v>
+      </c>
+      <c r="F9" t="n">
         <v>2</v>
       </c>
-      <c r="G33" t="n">
-        <v>5.4739</v>
-      </c>
-      <c r="H33" t="n">
+      <c r="G9" t="n">
+        <v>9.801299999999999</v>
+      </c>
+      <c r="H9" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>5.4906</v>
-      </c>
-      <c r="B34" t="n">
-        <v>2.0611</v>
-      </c>
-      <c r="C34" t="n">
-        <v>5.4906</v>
-      </c>
-      <c r="D34" t="n">
-        <v>2.4122</v>
-      </c>
-      <c r="E34" t="n">
-        <v>5.4906</v>
-      </c>
-      <c r="F34" t="n">
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9.8347</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2.046</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9.8347</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.2886</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9.8347</v>
+      </c>
+      <c r="F10" t="n">
         <v>2</v>
       </c>
-      <c r="G34" t="n">
-        <v>5.4906</v>
-      </c>
-      <c r="H34" t="n">
+      <c r="G10" t="n">
+        <v>9.8347</v>
+      </c>
+      <c r="H10" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>5.5072</v>
-      </c>
-      <c r="B35" t="n">
-        <v>2.0613</v>
-      </c>
-      <c r="C35" t="n">
-        <v>5.5072</v>
-      </c>
-      <c r="D35" t="n">
-        <v>2.4121</v>
-      </c>
-      <c r="E35" t="n">
-        <v>5.5072</v>
-      </c>
-      <c r="F35" t="n">
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9.868</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2.0474</v>
+      </c>
+      <c r="C11" t="n">
+        <v>9.868</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.2877</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9.868</v>
+      </c>
+      <c r="F11" t="n">
         <v>2</v>
       </c>
-      <c r="G35" t="n">
-        <v>5.5072</v>
-      </c>
-      <c r="H35" t="n">
+      <c r="G11" t="n">
+        <v>9.868</v>
+      </c>
+      <c r="H11" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>5.5239</v>
-      </c>
-      <c r="B36" t="n">
-        <v>2.0529</v>
-      </c>
-      <c r="C36" t="n">
-        <v>5.5239</v>
-      </c>
-      <c r="D36" t="n">
-        <v>2.4081</v>
-      </c>
-      <c r="E36" t="n">
-        <v>5.5239</v>
-      </c>
-      <c r="F36" t="n">
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9.901300000000001</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2.0433</v>
+      </c>
+      <c r="C12" t="n">
+        <v>9.901300000000001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.2866</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9.901300000000001</v>
+      </c>
+      <c r="F12" t="n">
         <v>2</v>
       </c>
-      <c r="G36" t="n">
-        <v>5.5239</v>
-      </c>
-      <c r="H36" t="n">
+      <c r="G12" t="n">
+        <v>9.901300000000001</v>
+      </c>
+      <c r="H12" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>5.5406</v>
-      </c>
-      <c r="B37" t="n">
-        <v>2.0593</v>
-      </c>
-      <c r="C37" t="n">
-        <v>5.5406</v>
-      </c>
-      <c r="D37" t="n">
-        <v>2.4086</v>
-      </c>
-      <c r="E37" t="n">
-        <v>5.5406</v>
-      </c>
-      <c r="F37" t="n">
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9.934699999999999</v>
+      </c>
+      <c r="B13" t="n">
+        <v>2.0445</v>
+      </c>
+      <c r="C13" t="n">
+        <v>9.934699999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.2872</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9.934699999999999</v>
+      </c>
+      <c r="F13" t="n">
         <v>2</v>
       </c>
-      <c r="G37" t="n">
-        <v>5.5406</v>
-      </c>
-      <c r="H37" t="n">
+      <c r="G13" t="n">
+        <v>9.934699999999999</v>
+      </c>
+      <c r="H13" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>5.5572</v>
-      </c>
-      <c r="B38" t="n">
-        <v>2.0596</v>
-      </c>
-      <c r="C38" t="n">
-        <v>5.5572</v>
-      </c>
-      <c r="D38" t="n">
-        <v>2.4096</v>
-      </c>
-      <c r="E38" t="n">
-        <v>5.5572</v>
-      </c>
-      <c r="F38" t="n">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>9.968</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2.0466</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9.968</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.2857</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9.968</v>
+      </c>
+      <c r="F14" t="n">
         <v>2</v>
       </c>
-      <c r="G38" t="n">
-        <v>5.5572</v>
-      </c>
-      <c r="H38" t="n">
+      <c r="G14" t="n">
+        <v>9.968</v>
+      </c>
+      <c r="H14" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>5.5739</v>
-      </c>
-      <c r="B39" t="n">
-        <v>2.0596</v>
-      </c>
-      <c r="C39" t="n">
-        <v>5.5739</v>
-      </c>
-      <c r="D39" t="n">
-        <v>2.4055</v>
-      </c>
-      <c r="E39" t="n">
-        <v>5.5739</v>
-      </c>
-      <c r="F39" t="n">
+    <row r="15">
+      <c r="A15" t="n">
+        <v>10.0013</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2.0448</v>
+      </c>
+      <c r="C15" t="n">
+        <v>10.0013</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.2888</v>
+      </c>
+      <c r="E15" t="n">
+        <v>10.0013</v>
+      </c>
+      <c r="F15" t="n">
         <v>2</v>
       </c>
-      <c r="G39" t="n">
-        <v>5.5739</v>
-      </c>
-      <c r="H39" t="n">
+      <c r="G15" t="n">
+        <v>10.0013</v>
+      </c>
+      <c r="H15" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>5.5906</v>
-      </c>
-      <c r="B40" t="n">
-        <v>2.0581</v>
-      </c>
-      <c r="C40" t="n">
-        <v>5.5906</v>
-      </c>
-      <c r="D40" t="n">
-        <v>2.4087</v>
-      </c>
-      <c r="E40" t="n">
-        <v>5.5906</v>
-      </c>
-      <c r="F40" t="n">
+    <row r="16">
+      <c r="C16" t="n">
+        <v>10.0347</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.2863</v>
+      </c>
+      <c r="E16" t="n">
+        <v>10.0347</v>
+      </c>
+      <c r="F16" t="n">
         <v>2</v>
       </c>
-      <c r="G40" t="n">
-        <v>5.5906</v>
-      </c>
-      <c r="H40" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>5.6072</v>
-      </c>
-      <c r="B41" t="n">
-        <v>2.0616</v>
-      </c>
-      <c r="C41" t="n">
-        <v>5.6072</v>
-      </c>
-      <c r="D41" t="n">
-        <v>2.408</v>
-      </c>
-      <c r="E41" t="n">
-        <v>5.6072</v>
-      </c>
-      <c r="F41" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" t="n">
-        <v>5.6072</v>
-      </c>
-      <c r="H41" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>5.6239</v>
-      </c>
-      <c r="B42" t="n">
-        <v>2.0598</v>
-      </c>
-      <c r="C42" t="n">
-        <v>5.6239</v>
-      </c>
-      <c r="D42" t="n">
-        <v>2.4078</v>
-      </c>
-      <c r="E42" t="n">
-        <v>5.6239</v>
-      </c>
-      <c r="F42" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" t="n">
-        <v>5.6239</v>
-      </c>
-      <c r="H42" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>5.6406</v>
-      </c>
-      <c r="B43" t="n">
-        <v>2.0622</v>
-      </c>
-      <c r="C43" t="n">
-        <v>5.6406</v>
-      </c>
-      <c r="D43" t="n">
-        <v>2.4048</v>
-      </c>
-      <c r="E43" t="n">
-        <v>5.6406</v>
-      </c>
-      <c r="F43" t="n">
-        <v>2</v>
-      </c>
-      <c r="G43" t="n">
-        <v>5.6406</v>
-      </c>
-      <c r="H43" t="n">
+      <c r="G16" t="n">
+        <v>10.0347</v>
+      </c>
+      <c r="H16" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fig.6/Fig.7 for FIO-Fast->Varmail 10 h (v4 2.185, robust 2.347, default 2.486) + xlsx; fix per-run clock in fig7-10h
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig7_10h.xlsx
+++ b/figs/data/fig7_10h.xlsx
@@ -228,12 +228,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'① OLTP 시작 OLTP 시작'!$C$2:$C$1</f>
+              <f>'① OLTP 시작 OLTP 시작'!$C$2:$C$31</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'① OLTP 시작 OLTP 시작'!$E$1:$D$1</f>
+              <f>'① OLTP 시작 OLTP 시작'!$D$2:$D$31</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -271,12 +271,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'① OLTP 시작 OLTP 시작'!$E$2:$E$29</f>
+              <f>'① OLTP 시작 OLTP 시작'!$E$2:$E$31</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'① OLTP 시작 OLTP 시작'!$F$2:$F$29</f>
+              <f>'① OLTP 시작 OLTP 시작'!$F$2:$F$31</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -318,7 +318,7 @@
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="1.6"/>
+          <max val="1.5"/>
           <min val="1.2"/>
         </scaling>
         <delete val="0"/>
@@ -725,12 +725,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'② 전환 직후 전환 직후'!$C$2:$C$1</f>
+              <f>'② 전환 직후 전환 직후'!$C$2:$C$25</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'② 전환 직후 전환 직후'!$E$1:$D$1</f>
+              <f>'② 전환 직후 전환 직후'!$D$2:$D$25</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -1222,12 +1222,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'③ 마지막 30분 마지막 30분'!$C$2:$C$1</f>
+              <f>'③ 마지막 30분 마지막 30분'!$C$2:$C$16</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'③ 마지막 30분 마지막 30분'!$E$1:$D$1</f>
+              <f>'③ 마지막 30분 마지막 30분'!$D$2:$D$16</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -1265,12 +1265,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'③ 마지막 30분 마지막 30분'!$E$2:$E$16</f>
+              <f>'③ 마지막 30분 마지막 30분'!$E$2:$E$15</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'③ 마지막 30분 마지막 30분'!$F$2:$F$16</f>
+              <f>'③ 마지막 30분 마지막 30분'!$F$2:$F$15</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -2190,11 +2190,17 @@
       <c r="B2" t="n">
         <v>1.3763</v>
       </c>
+      <c r="C2" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.3233</v>
+      </c>
       <c r="E2" t="n">
-        <v>0.0833</v>
+        <v>0.0167</v>
       </c>
       <c r="F2" t="n">
-        <v>1.5469</v>
+        <v>1.4909</v>
       </c>
       <c r="G2" t="n">
         <v>0.0167</v>
@@ -2219,11 +2225,17 @@
       <c r="B3" t="n">
         <v>1.2722</v>
       </c>
+      <c r="C3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.2684</v>
+      </c>
       <c r="E3" t="n">
-        <v>0.1167</v>
+        <v>0.05</v>
       </c>
       <c r="F3" t="n">
-        <v>1.4703</v>
+        <v>1.4522</v>
       </c>
       <c r="G3" t="n">
         <v>0.05</v>
@@ -2250,11 +2262,17 @@
       <c r="B4" t="n">
         <v>1.2803</v>
       </c>
+      <c r="C4" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.2574</v>
+      </c>
       <c r="E4" t="n">
-        <v>0.15</v>
+        <v>0.0833</v>
       </c>
       <c r="F4" t="n">
-        <v>1.447</v>
+        <v>1.4288</v>
       </c>
       <c r="G4" t="n">
         <v>0.0833</v>
@@ -2279,11 +2297,17 @@
       <c r="B5" t="n">
         <v>1.2616</v>
       </c>
+      <c r="C5" t="n">
+        <v>0.1167</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.2522</v>
+      </c>
       <c r="E5" t="n">
-        <v>0.1833</v>
+        <v>0.1167</v>
       </c>
       <c r="F5" t="n">
-        <v>1.4239</v>
+        <v>1.4113</v>
       </c>
       <c r="G5" t="n">
         <v>0.1167</v>
@@ -2305,11 +2329,17 @@
       <c r="B6" t="n">
         <v>1.2315</v>
       </c>
+      <c r="C6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.2482</v>
+      </c>
       <c r="E6" t="n">
-        <v>0.2167</v>
+        <v>0.15</v>
       </c>
       <c r="F6" t="n">
-        <v>1.4095</v>
+        <v>1.3999</v>
       </c>
       <c r="G6" t="n">
         <v>0.15</v>
@@ -2339,11 +2369,17 @@
       <c r="B7" t="n">
         <v>1.2334</v>
       </c>
+      <c r="C7" t="n">
+        <v>0.1833</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.2471</v>
+      </c>
       <c r="E7" t="n">
-        <v>0.25</v>
+        <v>0.1833</v>
       </c>
       <c r="F7" t="n">
-        <v>1.3949</v>
+        <v>1.3819</v>
       </c>
       <c r="G7" t="n">
         <v>0.1833</v>
@@ -2373,11 +2409,17 @@
       <c r="B8" t="n">
         <v>1.2304</v>
       </c>
+      <c r="C8" t="n">
+        <v>0.2167</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.243</v>
+      </c>
       <c r="E8" t="n">
-        <v>0.2833</v>
+        <v>0.2167</v>
       </c>
       <c r="F8" t="n">
-        <v>1.3764</v>
+        <v>1.3644</v>
       </c>
       <c r="G8" t="n">
         <v>0.2167</v>
@@ -2407,11 +2449,17 @@
       <c r="B9" t="n">
         <v>1.2243</v>
       </c>
+      <c r="C9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.2468</v>
+      </c>
       <c r="E9" t="n">
-        <v>0.3167</v>
+        <v>0.25</v>
       </c>
       <c r="F9" t="n">
-        <v>1.3627</v>
+        <v>1.3518</v>
       </c>
       <c r="G9" t="n">
         <v>0.25</v>
@@ -2433,11 +2481,17 @@
       <c r="B10" t="n">
         <v>1.2251</v>
       </c>
+      <c r="C10" t="n">
+        <v>0.2833</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.2449</v>
+      </c>
       <c r="E10" t="n">
-        <v>0.35</v>
+        <v>0.2833</v>
       </c>
       <c r="F10" t="n">
-        <v>1.3465</v>
+        <v>1.3388</v>
       </c>
       <c r="G10" t="n">
         <v>0.2833</v>
@@ -2459,11 +2513,17 @@
       <c r="B11" t="n">
         <v>1.2241</v>
       </c>
+      <c r="C11" t="n">
+        <v>0.3167</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.2452</v>
+      </c>
       <c r="E11" t="n">
-        <v>0.3833</v>
+        <v>0.3167</v>
       </c>
       <c r="F11" t="n">
-        <v>1.3363</v>
+        <v>1.3303</v>
       </c>
       <c r="G11" t="n">
         <v>0.3167</v>
@@ -2485,11 +2545,17 @@
       <c r="B12" t="n">
         <v>1.2214</v>
       </c>
+      <c r="C12" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.2435</v>
+      </c>
       <c r="E12" t="n">
-        <v>0.4167</v>
+        <v>0.35</v>
       </c>
       <c r="F12" t="n">
-        <v>1.3286</v>
+        <v>1.3249</v>
       </c>
       <c r="G12" t="n">
         <v>0.35</v>
@@ -2511,11 +2577,17 @@
       <c r="B13" t="n">
         <v>1.2232</v>
       </c>
+      <c r="C13" t="n">
+        <v>0.3833</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.2426</v>
+      </c>
       <c r="E13" t="n">
-        <v>0.45</v>
+        <v>0.3833</v>
       </c>
       <c r="F13" t="n">
-        <v>1.3231</v>
+        <v>1.3219</v>
       </c>
       <c r="G13" t="n">
         <v>0.3833</v>
@@ -2537,11 +2609,17 @@
       <c r="B14" t="n">
         <v>1.2224</v>
       </c>
+      <c r="C14" t="n">
+        <v>0.4167</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.2416</v>
+      </c>
       <c r="E14" t="n">
-        <v>0.4833</v>
+        <v>0.4167</v>
       </c>
       <c r="F14" t="n">
-        <v>1.3245</v>
+        <v>1.3208</v>
       </c>
       <c r="G14" t="n">
         <v>0.4167</v>
@@ -2563,11 +2641,17 @@
       <c r="B15" t="n">
         <v>1.2219</v>
       </c>
+      <c r="C15" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.241</v>
+      </c>
       <c r="E15" t="n">
-        <v>0.5167</v>
+        <v>0.45</v>
       </c>
       <c r="F15" t="n">
-        <v>1.3187</v>
+        <v>1.3165</v>
       </c>
       <c r="G15" t="n">
         <v>0.45</v>
@@ -2589,11 +2673,17 @@
       <c r="B16" t="n">
         <v>1.2208</v>
       </c>
+      <c r="C16" t="n">
+        <v>0.4833</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.2441</v>
+      </c>
       <c r="E16" t="n">
-        <v>0.55</v>
+        <v>0.4833</v>
       </c>
       <c r="F16" t="n">
-        <v>1.3152</v>
+        <v>1.3093</v>
       </c>
       <c r="G16" t="n">
         <v>0.4833</v>
@@ -2615,11 +2705,17 @@
       <c r="B17" t="n">
         <v>1.224</v>
       </c>
+      <c r="C17" t="n">
+        <v>0.5167</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.2427</v>
+      </c>
       <c r="E17" t="n">
-        <v>0.5833</v>
+        <v>0.5167</v>
       </c>
       <c r="F17" t="n">
-        <v>1.3087</v>
+        <v>1.3112</v>
       </c>
       <c r="G17" t="n">
         <v>0.5167</v>
@@ -2641,11 +2737,17 @@
       <c r="B18" t="n">
         <v>1.2219</v>
       </c>
+      <c r="C18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.241</v>
+      </c>
       <c r="E18" t="n">
-        <v>0.6167</v>
+        <v>0.55</v>
       </c>
       <c r="F18" t="n">
-        <v>1.3116</v>
+        <v>1.3128</v>
       </c>
       <c r="G18" t="n">
         <v>0.55</v>
@@ -2667,11 +2769,17 @@
       <c r="B19" t="n">
         <v>1.222</v>
       </c>
+      <c r="C19" t="n">
+        <v>0.5833</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.2416</v>
+      </c>
       <c r="E19" t="n">
-        <v>0.65</v>
+        <v>0.5833</v>
       </c>
       <c r="F19" t="n">
-        <v>1.3123</v>
+        <v>1.31</v>
       </c>
       <c r="G19" t="n">
         <v>0.5833</v>
@@ -2693,11 +2801,17 @@
       <c r="B20" t="n">
         <v>1.221</v>
       </c>
+      <c r="C20" t="n">
+        <v>0.6167</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1.2381</v>
+      </c>
       <c r="E20" t="n">
-        <v>0.6833</v>
+        <v>0.6167</v>
       </c>
       <c r="F20" t="n">
-        <v>1.3099</v>
+        <v>1.3087</v>
       </c>
       <c r="G20" t="n">
         <v>0.6167</v>
@@ -2719,11 +2833,17 @@
       <c r="B21" t="n">
         <v>1.2211</v>
       </c>
+      <c r="C21" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.2387</v>
+      </c>
       <c r="E21" t="n">
-        <v>0.7167</v>
+        <v>0.65</v>
       </c>
       <c r="F21" t="n">
-        <v>1.3083</v>
+        <v>1.3082</v>
       </c>
       <c r="G21" t="n">
         <v>0.65</v>
@@ -2745,11 +2865,17 @@
       <c r="B22" t="n">
         <v>1.2209</v>
       </c>
+      <c r="C22" t="n">
+        <v>0.6833</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.2389</v>
+      </c>
       <c r="E22" t="n">
-        <v>0.75</v>
+        <v>0.6833</v>
       </c>
       <c r="F22" t="n">
-        <v>1.3088</v>
+        <v>1.3071</v>
       </c>
       <c r="G22" t="n">
         <v>0.6833</v>
@@ -2771,11 +2897,17 @@
       <c r="B23" t="n">
         <v>1.2219</v>
       </c>
+      <c r="C23" t="n">
+        <v>0.7167</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.2396</v>
+      </c>
       <c r="E23" t="n">
-        <v>0.7833</v>
+        <v>0.7167</v>
       </c>
       <c r="F23" t="n">
-        <v>1.3072</v>
+        <v>1.3071</v>
       </c>
       <c r="G23" t="n">
         <v>0.7167</v>
@@ -2797,11 +2929,17 @@
       <c r="B24" t="n">
         <v>1.2241</v>
       </c>
+      <c r="C24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.2406</v>
+      </c>
       <c r="E24" t="n">
-        <v>0.8167</v>
+        <v>0.75</v>
       </c>
       <c r="F24" t="n">
-        <v>1.3072</v>
+        <v>1.3079</v>
       </c>
       <c r="G24" t="n">
         <v>0.75</v>
@@ -2823,11 +2961,17 @@
       <c r="B25" t="n">
         <v>1.2163</v>
       </c>
+      <c r="C25" t="n">
+        <v>0.7833</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1.2368</v>
+      </c>
       <c r="E25" t="n">
-        <v>0.85</v>
+        <v>0.7833</v>
       </c>
       <c r="F25" t="n">
-        <v>1.3055</v>
+        <v>1.3035</v>
       </c>
       <c r="G25" t="n">
         <v>0.7833</v>
@@ -2849,11 +2993,17 @@
       <c r="B26" t="n">
         <v>1.2212</v>
       </c>
+      <c r="C26" t="n">
+        <v>0.8167</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.2377</v>
+      </c>
       <c r="E26" t="n">
-        <v>0.8833</v>
+        <v>0.8167</v>
       </c>
       <c r="F26" t="n">
-        <v>1.3039</v>
+        <v>1.3022</v>
       </c>
       <c r="G26" t="n">
         <v>0.8167</v>
@@ -2875,11 +3025,17 @@
       <c r="B27" t="n">
         <v>1.2172</v>
       </c>
+      <c r="C27" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.2375</v>
+      </c>
       <c r="E27" t="n">
-        <v>0.9167</v>
+        <v>0.85</v>
       </c>
       <c r="F27" t="n">
-        <v>1.3021</v>
+        <v>1.3036</v>
       </c>
       <c r="G27" t="n">
         <v>0.85</v>
@@ -2901,11 +3057,17 @@
       <c r="B28" t="n">
         <v>1.2156</v>
       </c>
+      <c r="C28" t="n">
+        <v>0.8833</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.2372</v>
+      </c>
       <c r="E28" t="n">
-        <v>0.95</v>
+        <v>0.8833</v>
       </c>
       <c r="F28" t="n">
-        <v>1.3031</v>
+        <v>1.3024</v>
       </c>
       <c r="G28" t="n">
         <v>0.8833</v>
@@ -2927,11 +3089,17 @@
       <c r="B29" t="n">
         <v>1.2166</v>
       </c>
+      <c r="C29" t="n">
+        <v>0.9167</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.2384</v>
+      </c>
       <c r="E29" t="n">
-        <v>0.9833</v>
+        <v>0.9167</v>
       </c>
       <c r="F29" t="n">
-        <v>1.3026</v>
+        <v>1.3005</v>
       </c>
       <c r="G29" t="n">
         <v>0.9167</v>
@@ -2953,6 +3121,18 @@
       <c r="B30" t="n">
         <v>1.2143</v>
       </c>
+      <c r="C30" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.2362</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.3006</v>
+      </c>
       <c r="G30" t="n">
         <v>0.95</v>
       </c>
@@ -2972,6 +3152,18 @@
       </c>
       <c r="B31" t="n">
         <v>1.2151</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.9833</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.2376</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.9833</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.2999</v>
       </c>
       <c r="G31" t="n">
         <v>0.9833</v>
@@ -3065,11 +3257,17 @@
       <c r="B2" t="n">
         <v>1.227</v>
       </c>
+      <c r="C2" t="n">
+        <v>4.9656</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.2268</v>
+      </c>
       <c r="E2" t="n">
         <v>4.9656</v>
       </c>
       <c r="F2" t="n">
-        <v>1.2839</v>
+        <v>1.2818</v>
       </c>
       <c r="G2" t="n">
         <v>4.9656</v>
@@ -3094,11 +3292,17 @@
       <c r="B3" t="n">
         <v>1.2264</v>
       </c>
+      <c r="C3" t="n">
+        <v>4.9989</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.2253</v>
+      </c>
       <c r="E3" t="n">
         <v>4.9989</v>
       </c>
       <c r="F3" t="n">
-        <v>1.2816</v>
+        <v>1.2819</v>
       </c>
       <c r="G3" t="n">
         <v>4.9989</v>
@@ -3125,11 +3329,17 @@
       <c r="B4" t="n">
         <v>1.2263</v>
       </c>
+      <c r="C4" t="n">
+        <v>5.0322</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.226</v>
+      </c>
       <c r="E4" t="n">
         <v>5.0322</v>
       </c>
       <c r="F4" t="n">
-        <v>1.2805</v>
+        <v>2.2286</v>
       </c>
       <c r="G4" t="n">
         <v>5.0322</v>
@@ -3154,11 +3364,17 @@
       <c r="B5" t="n">
         <v>2.0441</v>
       </c>
+      <c r="C5" t="n">
+        <v>5.0656</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.8707</v>
+      </c>
       <c r="E5" t="n">
         <v>5.0656</v>
       </c>
       <c r="F5" t="n">
-        <v>1.2815</v>
+        <v>2.4242</v>
       </c>
       <c r="G5" t="n">
         <v>5.0656</v>
@@ -3180,11 +3396,17 @@
       <c r="B6" t="n">
         <v>2.0819</v>
       </c>
+      <c r="C6" t="n">
+        <v>5.0989</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.0437</v>
+      </c>
       <c r="E6" t="n">
         <v>5.0989</v>
       </c>
       <c r="F6" t="n">
-        <v>1.2852</v>
+        <v>2.4288</v>
       </c>
       <c r="G6" t="n">
         <v>5.0989</v>
@@ -3214,11 +3436,17 @@
       <c r="B7" t="n">
         <v>2.0839</v>
       </c>
+      <c r="C7" t="n">
+        <v>5.1322</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.051</v>
+      </c>
       <c r="E7" t="n">
         <v>5.1322</v>
       </c>
       <c r="F7" t="n">
-        <v>2.342</v>
+        <v>2.4276</v>
       </c>
       <c r="G7" t="n">
         <v>5.1322</v>
@@ -3248,11 +3476,17 @@
       <c r="B8" t="n">
         <v>2.0852</v>
       </c>
+      <c r="C8" t="n">
+        <v>5.1656</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.0508</v>
+      </c>
       <c r="E8" t="n">
         <v>5.1656</v>
       </c>
       <c r="F8" t="n">
-        <v>2.4259</v>
+        <v>2.4284</v>
       </c>
       <c r="G8" t="n">
         <v>5.1656</v>
@@ -3282,11 +3516,17 @@
       <c r="B9" t="n">
         <v>2.0764</v>
       </c>
+      <c r="C9" t="n">
+        <v>5.1989</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.0516</v>
+      </c>
       <c r="E9" t="n">
         <v>5.1989</v>
       </c>
       <c r="F9" t="n">
-        <v>2.428</v>
+        <v>2.4269</v>
       </c>
       <c r="G9" t="n">
         <v>5.1989</v>
@@ -3308,11 +3548,17 @@
       <c r="B10" t="n">
         <v>2.0724</v>
       </c>
+      <c r="C10" t="n">
+        <v>5.2322</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.0508</v>
+      </c>
       <c r="E10" t="n">
         <v>5.2322</v>
       </c>
       <c r="F10" t="n">
-        <v>2.4276</v>
+        <v>2.4242</v>
       </c>
       <c r="G10" t="n">
         <v>5.2322</v>
@@ -3334,11 +3580,17 @@
       <c r="B11" t="n">
         <v>2.0722</v>
       </c>
+      <c r="C11" t="n">
+        <v>5.2656</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.0504</v>
+      </c>
       <c r="E11" t="n">
         <v>5.2656</v>
       </c>
       <c r="F11" t="n">
-        <v>2.4287</v>
+        <v>2.4212</v>
       </c>
       <c r="G11" t="n">
         <v>5.2656</v>
@@ -3360,11 +3612,17 @@
       <c r="B12" t="n">
         <v>2.0748</v>
       </c>
+      <c r="C12" t="n">
+        <v>5.2989</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.0521</v>
+      </c>
       <c r="E12" t="n">
         <v>5.2989</v>
       </c>
       <c r="F12" t="n">
-        <v>2.4263</v>
+        <v>2.4228</v>
       </c>
       <c r="G12" t="n">
         <v>5.2989</v>
@@ -3386,11 +3644,17 @@
       <c r="B13" t="n">
         <v>2.0727</v>
       </c>
+      <c r="C13" t="n">
+        <v>5.3322</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.0503</v>
+      </c>
       <c r="E13" t="n">
         <v>5.3322</v>
       </c>
       <c r="F13" t="n">
-        <v>2.4228</v>
+        <v>2.4211</v>
       </c>
       <c r="G13" t="n">
         <v>5.3322</v>
@@ -3412,11 +3676,17 @@
       <c r="B14" t="n">
         <v>2.072</v>
       </c>
+      <c r="C14" t="n">
+        <v>5.3656</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.0524</v>
+      </c>
       <c r="E14" t="n">
         <v>5.3656</v>
       </c>
       <c r="F14" t="n">
-        <v>2.4221</v>
+        <v>2.4162</v>
       </c>
       <c r="G14" t="n">
         <v>5.3656</v>
@@ -3438,11 +3708,17 @@
       <c r="B15" t="n">
         <v>2.0679</v>
       </c>
+      <c r="C15" t="n">
+        <v>5.3989</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.053</v>
+      </c>
       <c r="E15" t="n">
         <v>5.3989</v>
       </c>
       <c r="F15" t="n">
-        <v>2.4225</v>
+        <v>2.4129</v>
       </c>
       <c r="G15" t="n">
         <v>5.3989</v>
@@ -3464,11 +3740,17 @@
       <c r="B16" t="n">
         <v>2.0594</v>
       </c>
+      <c r="C16" t="n">
+        <v>5.4322</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.0515</v>
+      </c>
       <c r="E16" t="n">
         <v>5.4322</v>
       </c>
       <c r="F16" t="n">
-        <v>2.4205</v>
+        <v>2.4095</v>
       </c>
       <c r="G16" t="n">
         <v>5.4322</v>
@@ -3490,11 +3772,17 @@
       <c r="B17" t="n">
         <v>2.0609</v>
       </c>
+      <c r="C17" t="n">
+        <v>5.4656</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.0513</v>
+      </c>
       <c r="E17" t="n">
         <v>5.4656</v>
       </c>
       <c r="F17" t="n">
-        <v>2.415</v>
+        <v>2.4083</v>
       </c>
       <c r="G17" t="n">
         <v>5.4656</v>
@@ -3516,11 +3804,17 @@
       <c r="B18" t="n">
         <v>2.0612</v>
       </c>
+      <c r="C18" t="n">
+        <v>5.4989</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.0517</v>
+      </c>
       <c r="E18" t="n">
         <v>5.4989</v>
       </c>
       <c r="F18" t="n">
-        <v>2.4122</v>
+        <v>2.4074</v>
       </c>
       <c r="G18" t="n">
         <v>5.4989</v>
@@ -3542,11 +3836,17 @@
       <c r="B19" t="n">
         <v>2.0562</v>
       </c>
+      <c r="C19" t="n">
+        <v>5.5322</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.0521</v>
+      </c>
       <c r="E19" t="n">
         <v>5.5322</v>
       </c>
       <c r="F19" t="n">
-        <v>2.4083</v>
+        <v>2.4072</v>
       </c>
       <c r="G19" t="n">
         <v>5.5322</v>
@@ -3568,11 +3868,17 @@
       <c r="B20" t="n">
         <v>2.0596</v>
       </c>
+      <c r="C20" t="n">
+        <v>5.5656</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.0499</v>
+      </c>
       <c r="E20" t="n">
         <v>5.5656</v>
       </c>
       <c r="F20" t="n">
-        <v>2.4076</v>
+        <v>2.4044</v>
       </c>
       <c r="G20" t="n">
         <v>5.5656</v>
@@ -3594,11 +3900,17 @@
       <c r="B21" t="n">
         <v>2.0599</v>
       </c>
+      <c r="C21" t="n">
+        <v>5.5989</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.0515</v>
+      </c>
       <c r="E21" t="n">
         <v>5.5989</v>
       </c>
       <c r="F21" t="n">
-        <v>2.4083</v>
+        <v>2.4012</v>
       </c>
       <c r="G21" t="n">
         <v>5.5989</v>
@@ -3620,11 +3932,17 @@
       <c r="B22" t="n">
         <v>2.061</v>
       </c>
+      <c r="C22" t="n">
+        <v>5.6322</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.0509</v>
+      </c>
       <c r="E22" t="n">
         <v>5.6322</v>
       </c>
       <c r="F22" t="n">
-        <v>2.4063</v>
+        <v>2.4022</v>
       </c>
       <c r="G22" t="n">
         <v>5.6322</v>
@@ -3646,11 +3964,17 @@
       <c r="B23" t="n">
         <v>2.0603</v>
       </c>
+      <c r="C23" t="n">
+        <v>5.6656</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2.0517</v>
+      </c>
       <c r="E23" t="n">
         <v>5.6656</v>
       </c>
       <c r="F23" t="n">
-        <v>2.4038</v>
+        <v>2.3991</v>
       </c>
       <c r="G23" t="n">
         <v>5.6656</v>
@@ -3672,11 +3996,17 @@
       <c r="B24" t="n">
         <v>2.0656</v>
       </c>
+      <c r="C24" t="n">
+        <v>5.6989</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2.051</v>
+      </c>
       <c r="E24" t="n">
         <v>5.6989</v>
       </c>
       <c r="F24" t="n">
-        <v>2.4013</v>
+        <v>2.3965</v>
       </c>
       <c r="G24" t="n">
         <v>5.6989</v>
@@ -3698,11 +4028,17 @@
       <c r="B25" t="n">
         <v>2.0633</v>
       </c>
+      <c r="C25" t="n">
+        <v>5.7322</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2.0509</v>
+      </c>
       <c r="E25" t="n">
         <v>5.7322</v>
       </c>
       <c r="F25" t="n">
-        <v>2.4026</v>
+        <v>2.3939</v>
       </c>
       <c r="G25" t="n">
         <v>5.7322</v>
@@ -3796,11 +4132,17 @@
       <c r="B2" t="n">
         <v>2.0458</v>
       </c>
+      <c r="C2" t="n">
+        <v>9.568</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.0508</v>
+      </c>
       <c r="E2" t="n">
         <v>9.568</v>
       </c>
       <c r="F2" t="n">
-        <v>2.2932</v>
+        <v>2.2912</v>
       </c>
       <c r="G2" t="n">
         <v>9.568</v>
@@ -3825,11 +4167,17 @@
       <c r="B3" t="n">
         <v>2.0457</v>
       </c>
+      <c r="C3" t="n">
+        <v>9.6013</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.0513</v>
+      </c>
       <c r="E3" t="n">
         <v>9.6013</v>
       </c>
       <c r="F3" t="n">
-        <v>2.2907</v>
+        <v>2.2912</v>
       </c>
       <c r="G3" t="n">
         <v>9.6013</v>
@@ -3856,11 +4204,17 @@
       <c r="B4" t="n">
         <v>2.0466</v>
       </c>
+      <c r="C4" t="n">
+        <v>9.6347</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.051</v>
+      </c>
       <c r="E4" t="n">
         <v>9.6347</v>
       </c>
       <c r="F4" t="n">
-        <v>2.2924</v>
+        <v>2.2908</v>
       </c>
       <c r="G4" t="n">
         <v>9.6347</v>
@@ -3885,11 +4239,17 @@
       <c r="B5" t="n">
         <v>2.0452</v>
       </c>
+      <c r="C5" t="n">
+        <v>9.667999999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.0519</v>
+      </c>
       <c r="E5" t="n">
         <v>9.667999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>2.2915</v>
+        <v>2.2899</v>
       </c>
       <c r="G5" t="n">
         <v>9.667999999999999</v>
@@ -3911,11 +4271,17 @@
       <c r="B6" t="n">
         <v>2.0466</v>
       </c>
+      <c r="C6" t="n">
+        <v>9.7013</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.0497</v>
+      </c>
       <c r="E6" t="n">
         <v>9.7013</v>
       </c>
       <c r="F6" t="n">
-        <v>2.2914</v>
+        <v>2.289</v>
       </c>
       <c r="G6" t="n">
         <v>9.7013</v>
@@ -3945,11 +4311,17 @@
       <c r="B7" t="n">
         <v>2.0458</v>
       </c>
+      <c r="C7" t="n">
+        <v>9.7347</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.0502</v>
+      </c>
       <c r="E7" t="n">
         <v>9.7347</v>
       </c>
       <c r="F7" t="n">
-        <v>2.2906</v>
+        <v>2.2874</v>
       </c>
       <c r="G7" t="n">
         <v>9.7347</v>
@@ -3979,11 +4351,17 @@
       <c r="B8" t="n">
         <v>2.045</v>
       </c>
+      <c r="C8" t="n">
+        <v>9.768000000000001</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.0515</v>
+      </c>
       <c r="E8" t="n">
         <v>9.768000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>2.2894</v>
+        <v>2.2877</v>
       </c>
       <c r="G8" t="n">
         <v>9.768000000000001</v>
@@ -4013,11 +4391,17 @@
       <c r="B9" t="n">
         <v>2.0434</v>
       </c>
+      <c r="C9" t="n">
+        <v>9.801299999999999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.0492</v>
+      </c>
       <c r="E9" t="n">
         <v>9.801299999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>2.2884</v>
+        <v>2.288</v>
       </c>
       <c r="G9" t="n">
         <v>9.801299999999999</v>
@@ -4039,11 +4423,17 @@
       <c r="B10" t="n">
         <v>2.046</v>
       </c>
+      <c r="C10" t="n">
+        <v>9.8347</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.0497</v>
+      </c>
       <c r="E10" t="n">
         <v>9.8347</v>
       </c>
       <c r="F10" t="n">
-        <v>2.2886</v>
+        <v>2.2869</v>
       </c>
       <c r="G10" t="n">
         <v>9.8347</v>
@@ -4065,11 +4455,17 @@
       <c r="B11" t="n">
         <v>2.0474</v>
       </c>
+      <c r="C11" t="n">
+        <v>9.868</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.05</v>
+      </c>
       <c r="E11" t="n">
         <v>9.868</v>
       </c>
       <c r="F11" t="n">
-        <v>2.2877</v>
+        <v>2.2865</v>
       </c>
       <c r="G11" t="n">
         <v>9.868</v>
@@ -4091,11 +4487,17 @@
       <c r="B12" t="n">
         <v>2.0433</v>
       </c>
+      <c r="C12" t="n">
+        <v>9.901300000000001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.05</v>
+      </c>
       <c r="E12" t="n">
         <v>9.901300000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>2.2866</v>
+        <v>2.2871</v>
       </c>
       <c r="G12" t="n">
         <v>9.901300000000001</v>
@@ -4117,11 +4519,17 @@
       <c r="B13" t="n">
         <v>2.0445</v>
       </c>
+      <c r="C13" t="n">
+        <v>9.934699999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.0509</v>
+      </c>
       <c r="E13" t="n">
         <v>9.934699999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>2.2872</v>
+        <v>2.2877</v>
       </c>
       <c r="G13" t="n">
         <v>9.934699999999999</v>
@@ -4143,11 +4551,17 @@
       <c r="B14" t="n">
         <v>2.0466</v>
       </c>
+      <c r="C14" t="n">
+        <v>9.968</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.0495</v>
+      </c>
       <c r="E14" t="n">
         <v>9.968</v>
       </c>
       <c r="F14" t="n">
-        <v>2.2857</v>
+        <v>2.2861</v>
       </c>
       <c r="G14" t="n">
         <v>9.968</v>
@@ -4169,11 +4583,17 @@
       <c r="B15" t="n">
         <v>2.0448</v>
       </c>
+      <c r="C15" t="n">
+        <v>10.0013</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.0506</v>
+      </c>
       <c r="E15" t="n">
         <v>10.0013</v>
       </c>
       <c r="F15" t="n">
-        <v>2.2888</v>
+        <v>2.2857</v>
       </c>
       <c r="G15" t="n">
         <v>10.0013</v>
@@ -4189,11 +4609,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="E16" t="n">
+      <c r="C16" t="n">
         <v>10.0347</v>
       </c>
-      <c r="F16" t="n">
-        <v>2.2863</v>
+      <c r="D16" t="n">
+        <v>2.0503</v>
       </c>
       <c r="G16" t="n">
         <v>10.0347</v>

</xml_diff>